<commit_message>
Finished first draft of MLP hyperparameter tuning
</commit_message>
<xml_diff>
--- a/results/models_performance.xlsx
+++ b/results/models_performance.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -715,128 +715,128 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HISTMEAN</t>
+          <t>MLP_step_aug_TPE</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12.802</v>
+        <v>2.6272</v>
       </c>
       <c r="D14" t="n">
-        <v>11.8563</v>
+        <v>2.3462</v>
       </c>
       <c r="E14" t="n">
-        <v>12.2</v>
+        <v>2.48</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Employment in agriculture (% of total employment)</t>
+          <t>Crop production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HISTMEAN</t>
+          <t>MLP_jitter_aug_Random</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1.1843</v>
+        <v>3.3793</v>
       </c>
       <c r="D15" t="n">
-        <v>1.1758</v>
+        <v>2.3761</v>
       </c>
       <c r="E15" t="n">
-        <v>30.84</v>
+        <v>2.47</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Employment in agriculture, female (% of female employment)</t>
+          <t>Crop production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HISTMEAN</t>
+          <t>MLP_step_aug_Random</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1.8927</v>
+        <v>3.5746</v>
       </c>
       <c r="D16" t="n">
-        <v>1.8909</v>
+        <v>3.3431</v>
       </c>
       <c r="E16" t="n">
-        <v>80.34999999999999</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Employment in agriculture, male (% of male employment)</t>
+          <t>Crop production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HISTMEAN</t>
+          <t>MLP_jitter_aug_TPE</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.6382</v>
+        <v>4.1733</v>
       </c>
       <c r="D17" t="n">
-        <v>0.61</v>
+        <v>3.1882</v>
       </c>
       <c r="E17" t="n">
-        <v>12.61</v>
+        <v>3.32</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Crop production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>HISTMEAN</t>
+          <t>MLP_orig_Random</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>89.9853</v>
+        <v>9.039300000000001</v>
       </c>
       <c r="D18" t="n">
-        <v>74.8262</v>
+        <v>8.9551</v>
       </c>
       <c r="E18" t="n">
-        <v>38.99</v>
+        <v>9.44</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Crop production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HISTMEAN</t>
+          <t>MLP_orig_TPE</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>49.5005</v>
+        <v>10.4076</v>
       </c>
       <c r="D19" t="n">
-        <v>49.0597</v>
+        <v>10.316</v>
       </c>
       <c r="E19" t="n">
-        <v>39.16</v>
+        <v>10.83</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Food production index (2014-2016 = 100)</t>
+          <t>Crop production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -845,19 +845,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>6.2587</v>
+        <v>12.802</v>
       </c>
       <c r="D20" t="n">
-        <v>5.671</v>
+        <v>11.8563</v>
       </c>
       <c r="E20" t="n">
-        <v>5.71</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Forest area (% of land area)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -866,19 +866,19 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>3.3816</v>
+        <v>1.1843</v>
       </c>
       <c r="D21" t="n">
-        <v>3.3619</v>
+        <v>1.1758</v>
       </c>
       <c r="E21" t="n">
-        <v>10.44</v>
+        <v>30.84</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Forest area (sq. km)</t>
+          <t>Employment in agriculture, female (% of female employment)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,19 +887,19 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>10165.8396</v>
+        <v>1.8927</v>
       </c>
       <c r="D22" t="n">
-        <v>10108.7135</v>
+        <v>1.8909</v>
       </c>
       <c r="E22" t="n">
-        <v>10.62</v>
+        <v>80.34999999999999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Land under cereal production (hectares)</t>
+          <t>Employment in agriculture, male (% of male employment)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -908,19 +908,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1645417.9467</v>
+        <v>0.6382</v>
       </c>
       <c r="D23" t="n">
-        <v>1634397.1444</v>
+        <v>0.61</v>
       </c>
       <c r="E23" t="n">
-        <v>50.99</v>
+        <v>12.61</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Livestock production index (2014-2016 = 100)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -929,19 +929,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>7.9306</v>
+        <v>89.9853</v>
       </c>
       <c r="D24" t="n">
-        <v>7.2338</v>
+        <v>74.8262</v>
       </c>
       <c r="E24" t="n">
-        <v>6.83</v>
+        <v>38.99</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Permanent cropland (% of land area)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -950,19 +950,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.5853</v>
+        <v>49.5005</v>
       </c>
       <c r="D25" t="n">
-        <v>1.5333</v>
+        <v>49.0597</v>
       </c>
       <c r="E25" t="n">
-        <v>19.21</v>
+        <v>39.16</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rural population</t>
+          <t>Food production index (2014-2016 = 100)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -971,19 +971,19 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1620364.5486</v>
+        <v>6.2587</v>
       </c>
       <c r="D26" t="n">
-        <v>1400345.8654</v>
+        <v>5.671</v>
       </c>
       <c r="E26" t="n">
-        <v>8.17</v>
+        <v>5.71</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Forest area (% of land area)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -992,33 +992,159 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>4.7939</v>
+        <v>3.3816</v>
       </c>
       <c r="D27" t="n">
-        <v>4.6613</v>
+        <v>3.3619</v>
       </c>
       <c r="E27" t="n">
-        <v>15.95</v>
+        <v>10.44</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>Forest area (sq. km)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>10165.8396</v>
+      </c>
+      <c r="D28" t="n">
+        <v>10108.7135</v>
+      </c>
+      <c r="E28" t="n">
+        <v>10.62</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Land under cereal production (hectares)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>1645417.9467</v>
+      </c>
+      <c r="D29" t="n">
+        <v>1634397.1444</v>
+      </c>
+      <c r="E29" t="n">
+        <v>50.99</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>7.9306</v>
+      </c>
+      <c r="D30" t="n">
+        <v>7.2338</v>
+      </c>
+      <c r="E30" t="n">
+        <v>6.83</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Permanent cropland (% of land area)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1.5853</v>
+      </c>
+      <c r="D31" t="n">
+        <v>1.5333</v>
+      </c>
+      <c r="E31" t="n">
+        <v>19.21</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Rural population</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>1620364.5486</v>
+      </c>
+      <c r="D32" t="n">
+        <v>1400345.8654</v>
+      </c>
+      <c r="E32" t="n">
+        <v>8.17</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>4.7939</v>
+      </c>
+      <c r="D33" t="n">
+        <v>4.6613</v>
+      </c>
+      <c r="E33" t="n">
+        <v>15.95</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Rural population growth (annual %)</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>HISTMEAN</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HISTMEAN</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
         <v>1.0451</v>
       </c>
-      <c r="D28" t="n">
+      <c r="D34" t="n">
         <v>0.9893999999999999</v>
       </c>
-      <c r="E28" t="n">
+      <c r="E34" t="n">
         <v>85.67</v>
       </c>
     </row>

</xml_diff>